<commit_message>
added full_adder_1b_optimized macro which uses the minimal 9 NAND gates, making memory usage significantly more efficient.
</commit_message>
<xml_diff>
--- a/OneGatePython/memory_map.xlsx
+++ b/OneGatePython/memory_map.xlsx
@@ -901,13 +901,13 @@
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr"/>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr"/>
+      <c r="D10" s="11" t="inlineStr"/>
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>scratch</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr"/>
-      <c r="E10" s="11" t="inlineStr"/>
       <c r="F10" s="11" t="inlineStr"/>
       <c r="G10" s="11" t="inlineStr"/>
       <c r="H10" s="11" t="inlineStr"/>

</xml_diff>